<commit_message>
Hoan thien theo gop y 15/10: CTDT 2026, de cuong, nhap diem, gop bai, phu dao, de giay + cham phieu, dong bo cau hoi; kiem thu toan bo (24/10/2026)
</commit_message>
<xml_diff>
--- a/docs/kiem_thu/KET_QUA_KIEM_THU.xlsx
+++ b/docs/kiem_thu/KET_QUA_KIEM_THU.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -491,14 +491,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thời điểm chạy: 24/10/2026 10:06 · Python 3.13.17 · CSDL: kiểm thử dựng lại assessment_db</t>
+          <t>Thời điểm chạy: 24/10/2026 20:08 · Python 3.13.17 · CSDL: kiểm thử dựng lại assessment_db</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Ca kiểm thử tự động: 112/112 đạt · Độ phủ API: 137/138 endpoint được gọi thành công</t>
+          <t>Ca kiểm thử tự động: 129/129 đạt · Độ phủ API: 147/148 endpoint được gọi thành công</t>
         </is>
       </c>
     </row>
@@ -788,10 +788,10 @@
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D18" s="4" t="n">
         <v>0</v>
@@ -805,14 +805,14 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>TỔNG</t>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>112</v>
+        <v>25</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>112</v>
+        <v>25</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>0</v>
@@ -823,8 +823,29 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>TỔNG</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>129</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>129</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Kiểm thử bổ sung (ngoài pytest): tools/moodle_e2e/run_real_moodle_e2e.py (Moodle 4.5 thật), tools/moodle_e2e/kiem_tra_dong_bo_cau_hoi.py, tools/kiem_tra_do_luong.py (tính lại độc lập các độ đo), tools/omr/kiem_tra_omr.py (độ bền chấm phiếu), backend/tests/ui_screens.py (duyệt giao diện).</t>
         </is>
@@ -841,7 +862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I113"/>
+  <dimension ref="A1:I130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -932,7 +953,7 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>15.76</v>
+        <v>22.52</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
@@ -971,7 +992,7 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.1</v>
+        <v>0.26</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
@@ -1010,7 +1031,7 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.09</v>
+        <v>0.16</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
@@ -1049,7 +1070,7 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
@@ -1088,7 +1109,7 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
@@ -1127,7 +1148,7 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
@@ -1244,7 +1265,7 @@
         </is>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
@@ -1283,7 +1304,7 @@
         </is>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
@@ -1361,7 +1382,7 @@
         </is>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.09</v>
+        <v>0.14</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
@@ -1400,7 +1421,7 @@
         </is>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
@@ -1478,7 +1499,7 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.41</v>
+        <v>0.16</v>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
@@ -1595,7 +1616,7 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
@@ -1634,7 +1655,7 @@
         </is>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.09</v>
+        <v>0.13</v>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
@@ -1673,7 +1694,7 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
@@ -1868,7 +1889,7 @@
         </is>
       </c>
       <c r="G26" s="4" t="n">
-        <v>0.44</v>
+        <v>0.47</v>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
@@ -1985,7 +2006,7 @@
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
@@ -2063,7 +2084,7 @@
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.22</v>
+        <v>0.29</v>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
@@ -2258,7 +2279,7 @@
         </is>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
@@ -2297,7 +2318,7 @@
         </is>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.29</v>
+        <v>0.26</v>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
@@ -2336,7 +2357,7 @@
         </is>
       </c>
       <c r="G38" s="4" t="n">
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
@@ -2375,7 +2396,7 @@
         </is>
       </c>
       <c r="G39" s="4" t="n">
-        <v>0.28</v>
+        <v>0.25</v>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
@@ -2531,7 +2552,7 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>8.220000000000001</v>
+        <v>11.33</v>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
@@ -2570,7 +2591,7 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>16.82</v>
+        <v>21.8</v>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
@@ -2609,7 +2630,7 @@
         </is>
       </c>
       <c r="G45" s="4" t="n">
-        <v>8.56</v>
+        <v>11.35</v>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
@@ -2804,7 +2825,7 @@
         </is>
       </c>
       <c r="G50" s="4" t="n">
-        <v>4.54</v>
+        <v>6.05</v>
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
@@ -2843,7 +2864,7 @@
         </is>
       </c>
       <c r="G51" s="4" t="n">
-        <v>0.37</v>
+        <v>0.75</v>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
@@ -2921,7 +2942,7 @@
         </is>
       </c>
       <c r="G53" s="4" t="n">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
@@ -3350,7 +3371,7 @@
         </is>
       </c>
       <c r="G64" s="4" t="n">
-        <v>1.19</v>
+        <v>2.59</v>
       </c>
       <c r="H64" s="4" t="inlineStr">
         <is>
@@ -3428,7 +3449,7 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="H66" s="4" t="inlineStr">
         <is>
@@ -3467,7 +3488,7 @@
         </is>
       </c>
       <c r="G67" s="4" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
@@ -3506,7 +3527,7 @@
         </is>
       </c>
       <c r="G68" s="4" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="H68" s="4" t="inlineStr">
         <is>
@@ -3545,7 +3566,7 @@
         </is>
       </c>
       <c r="G69" s="4" t="n">
-        <v>0.45</v>
+        <v>0.28</v>
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
@@ -3584,7 +3605,7 @@
         </is>
       </c>
       <c r="G70" s="4" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="H70" s="4" t="inlineStr">
         <is>
@@ -3623,7 +3644,7 @@
         </is>
       </c>
       <c r="G71" s="4" t="n">
-        <v>1.1</v>
+        <v>1.25</v>
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
@@ -3662,7 +3683,7 @@
         </is>
       </c>
       <c r="G72" s="4" t="n">
-        <v>0.13</v>
+        <v>0.04</v>
       </c>
       <c r="H72" s="4" t="inlineStr">
         <is>
@@ -3701,7 +3722,7 @@
         </is>
       </c>
       <c r="G73" s="4" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
@@ -3779,7 +3800,7 @@
         </is>
       </c>
       <c r="G75" s="4" t="n">
-        <v>0.74</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
@@ -3818,7 +3839,7 @@
         </is>
       </c>
       <c r="G76" s="4" t="n">
-        <v>0.23</v>
+        <v>0.28</v>
       </c>
       <c r="H76" s="4" t="inlineStr">
         <is>
@@ -3857,7 +3878,7 @@
         </is>
       </c>
       <c r="G77" s="4" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
@@ -3896,7 +3917,7 @@
         </is>
       </c>
       <c r="G78" s="4" t="n">
-        <v>0.22</v>
+        <v>0.27</v>
       </c>
       <c r="H78" s="4" t="inlineStr">
         <is>
@@ -3974,7 +3995,7 @@
         </is>
       </c>
       <c r="G80" s="4" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="H80" s="4" t="inlineStr">
         <is>
@@ -4052,7 +4073,7 @@
         </is>
       </c>
       <c r="G82" s="4" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="H82" s="4" t="inlineStr">
         <is>
@@ -4091,7 +4112,7 @@
         </is>
       </c>
       <c r="G83" s="4" t="n">
-        <v>1.93</v>
+        <v>2.72</v>
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
@@ -4130,7 +4151,7 @@
         </is>
       </c>
       <c r="G84" s="4" t="n">
-        <v>0.13</v>
+        <v>0.21</v>
       </c>
       <c r="H84" s="4" t="inlineStr">
         <is>
@@ -4169,7 +4190,7 @@
         </is>
       </c>
       <c r="G85" s="4" t="n">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="H85" s="4" t="inlineStr">
         <is>
@@ -4208,7 +4229,7 @@
         </is>
       </c>
       <c r="G86" s="4" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="H86" s="4" t="inlineStr">
         <is>
@@ -4442,7 +4463,7 @@
         </is>
       </c>
       <c r="G92" s="4" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="H92" s="4" t="inlineStr">
         <is>
@@ -4481,7 +4502,7 @@
         </is>
       </c>
       <c r="G93" s="4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.14</v>
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
@@ -4559,7 +4580,7 @@
         </is>
       </c>
       <c r="G95" s="4" t="n">
-        <v>0.35</v>
+        <v>0.31</v>
       </c>
       <c r="H95" s="4" t="inlineStr">
         <is>
@@ -4598,7 +4619,7 @@
         </is>
       </c>
       <c r="G96" s="4" t="n">
-        <v>0.83</v>
+        <v>0.8</v>
       </c>
       <c r="H96" s="4" t="inlineStr">
         <is>
@@ -4637,7 +4658,7 @@
         </is>
       </c>
       <c r="G97" s="4" t="n">
-        <v>0.2</v>
+        <v>0.26</v>
       </c>
       <c r="H97" s="4" t="inlineStr">
         <is>
@@ -4676,7 +4697,7 @@
         </is>
       </c>
       <c r="G98" s="4" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="H98" s="4" t="inlineStr">
         <is>
@@ -4715,7 +4736,7 @@
         </is>
       </c>
       <c r="G99" s="4" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="H99" s="4" t="inlineStr">
         <is>
@@ -4793,7 +4814,7 @@
         </is>
       </c>
       <c r="G101" s="4" t="n">
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
       <c r="H101" s="4" t="inlineStr">
         <is>
@@ -4813,11 +4834,19 @@
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>test_seed_backfilled_clo_pi</t>
-        </is>
-      </c>
-      <c r="D102" s="4" t="inlineStr"/>
-      <c r="E102" s="4" t="inlineStr"/>
+          <t>Tính thời gian trả lời từng câu</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>Dãy thời điểm chọn đáp án; nhiều câu cùng một trang (cùng thời điểm)</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>Thời gian = khoảng cách tới lần chọn trước; câu cùng trang chia đều; báo độ phân giải theo trang</t>
+        </is>
+      </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
           <t>ĐẠT</t>
@@ -4828,7 +4857,7 @@
       </c>
       <c r="H102" s="4" t="inlineStr">
         <is>
-          <t>test_clo_pi::test_seed_backfilled_clo_pi</t>
+          <t>test_timing::test_response_time_split_and_page_resolution</t>
         </is>
       </c>
       <c r="I102" s="4" t="inlineStr"/>
@@ -4844,22 +4873,30 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>test_clo_pi_mapping_derives_plo</t>
-        </is>
-      </c>
-      <c r="D103" s="4" t="inlineStr"/>
-      <c r="E103" s="4" t="inlineStr"/>
+          <t>Đồng bộ thời điểm chọn đáp án từ Moodle</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>Đồng bộ Quiz có giới hạn 45 phút, tự nộp khi hết giờ</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="inlineStr">
+        <is>
+          <t>Lưu lần chọn đầu/cuối, số lần lưu từng câu; giới hạn thời gian; lượt hết giờ tự nộp</t>
+        </is>
+      </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
           <t>ĐẠT</t>
         </is>
       </c>
       <c r="G103" s="4" t="n">
-        <v>0.11</v>
+        <v>0.01</v>
       </c>
       <c r="H103" s="4" t="inlineStr">
         <is>
-          <t>test_clo_pi::test_clo_pi_mapping_derives_plo</t>
+          <t>test_timing::test_sync_stores_answer_times</t>
         </is>
       </c>
       <c r="I103" s="4" t="inlineStr"/>
@@ -4875,22 +4912,30 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>test_backfill_from_legacy_plo</t>
-        </is>
-      </c>
-      <c r="D104" s="4" t="inlineStr"/>
-      <c r="E104" s="4" t="inlineStr"/>
+          <t>Cảnh báo SV chọn đại / chọn xong để hết giờ</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>Dữ liệu có 2 SV chọn ~20 câu trong 1 phút và 2 SV chọn xong không nộp chờ hết giờ</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>Đúng 4 SV bị cảnh báo đúng loại; SV bình thường không bị gắn cờ; số cảnh báo hiện ở danh sách bài KT</t>
+        </is>
+      </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
           <t>ĐẠT</t>
         </is>
       </c>
       <c r="G104" s="4" t="n">
-        <v>0.03</v>
+        <v>0.41</v>
       </c>
       <c r="H104" s="4" t="inlineStr">
         <is>
-          <t>test_clo_pi::test_backfill_from_legacy_plo</t>
+          <t>test_timing::test_timing_report_flags_planted_students</t>
         </is>
       </c>
       <c r="I104" s="4" t="inlineStr"/>
@@ -4906,22 +4951,30 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>test_question_outcome_tree</t>
-        </is>
-      </c>
-      <c r="D105" s="4" t="inlineStr"/>
-      <c r="E105" s="4" t="inlineStr"/>
+          <t>Đổi ngưỡng, diễn biến từng SV, xuất Excel</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>Gửi ngưỡng tùy chỉnh / sai; xem diễn biến 1 SV; tải Excel; bài giấy</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>Kết quả theo ngưỡng; ngưỡng sai 422; SV không làm 404; Excel 2 sheet; bài giấy báo không áp dụng</t>
+        </is>
+      </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
           <t>ĐẠT</t>
         </is>
       </c>
       <c r="G105" s="4" t="n">
-        <v>0.12</v>
+        <v>0.24</v>
       </c>
       <c r="H105" s="4" t="inlineStr">
         <is>
-          <t>test_clo_pi::test_question_outcome_tree</t>
+          <t>test_timing::test_timing_thresholds_timeline_and_export</t>
         </is>
       </c>
       <c r="I105" s="4" t="inlineStr"/>
@@ -4932,12 +4985,12 @@
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>13. Thời gian làm bài &amp; cảnh báo bất thường</t>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>test_demo_syllabus_approved</t>
+          <t>test_seed_backfilled_clo_pi</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr"/>
@@ -4948,11 +5001,11 @@
         </is>
       </c>
       <c r="G106" s="4" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="H106" s="4" t="inlineStr">
         <is>
-          <t>test_syllabus_versions::test_demo_syllabus_approved</t>
+          <t>test_clo_pi::test_seed_backfilled_clo_pi</t>
         </is>
       </c>
       <c r="I106" s="4" t="inlineStr"/>
@@ -4963,12 +5016,12 @@
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>13. Thời gian làm bài &amp; cảnh báo bất thường</t>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>test_syllabus_version_flow</t>
+          <t>test_clo_pi_mapping_derives_plo</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr"/>
@@ -4979,11 +5032,11 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>0.38</v>
+        <v>0.14</v>
       </c>
       <c r="H107" s="4" t="inlineStr">
         <is>
-          <t>test_syllabus_versions::test_syllabus_version_flow</t>
+          <t>test_clo_pi::test_clo_pi_mapping_derives_plo</t>
         </is>
       </c>
       <c r="I107" s="4" t="inlineStr"/>
@@ -4994,12 +5047,12 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>13. Thời gian làm bài &amp; cảnh báo bất thường</t>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>test_outline_detail</t>
+          <t>test_backfill_from_legacy_plo</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr"/>
@@ -5010,11 +5063,11 @@
         </is>
       </c>
       <c r="G108" s="4" t="n">
-        <v>0.12</v>
+        <v>0.03</v>
       </c>
       <c r="H108" s="4" t="inlineStr">
         <is>
-          <t>test_syllabus_versions::test_outline_detail</t>
+          <t>test_clo_pi::test_backfill_from_legacy_plo</t>
         </is>
       </c>
       <c r="I108" s="4" t="inlineStr"/>
@@ -5025,12 +5078,12 @@
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>13. Thời gian làm bài &amp; cảnh báo bất thường</t>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>test_new_course_without_syllabus</t>
+          <t>test_question_outcome_tree</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr"/>
@@ -5041,11 +5094,11 @@
         </is>
       </c>
       <c r="G109" s="4" t="n">
-        <v>0.06</v>
+        <v>0.13</v>
       </c>
       <c r="H109" s="4" t="inlineStr">
         <is>
-          <t>test_syllabus_versions::test_new_course_without_syllabus</t>
+          <t>test_clo_pi::test_question_outcome_tree</t>
         </is>
       </c>
       <c r="I109" s="4" t="inlineStr"/>
@@ -5056,22 +5109,22 @@
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>13. Thời gian làm bài &amp; cảnh báo bất thường</t>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Tính thời gian trả lời từng câu</t>
+          <t>Học liệu mẫu có sẵn</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Dãy thời điểm chọn đáp án; nhiều câu cùng một trang (cùng thời điểm)</t>
+          <t>Danh sách học liệu của môn DBMS330284</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>Thời gian = khoảng cách tới lần chọn trước; câu cùng trang chia đều; báo độ phân giải theo trang</t>
+          <t>7 học liệu (6 slide + 1 giáo trình), số trang khớp nội dung đã sinh</t>
         </is>
       </c>
       <c r="F110" s="5" t="inlineStr">
@@ -5080,11 +5133,11 @@
         </is>
       </c>
       <c r="G110" s="4" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H110" s="4" t="inlineStr">
         <is>
-          <t>test_timing::test_response_time_split_and_page_resolution</t>
+          <t>test_hoc_lieu_rag::test_seed_co_hoc_lieu</t>
         </is>
       </c>
       <c r="I110" s="4" t="inlineStr"/>
@@ -5095,24 +5148,16 @@
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>13. Thời gian làm bài &amp; cảnh báo bất thường</t>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Đồng bộ thời điểm chọn đáp án từ Moodle</t>
-        </is>
-      </c>
-      <c r="D111" s="4" t="inlineStr">
-        <is>
-          <t>Đồng bộ Quiz có giới hạn 45 phút, tự nộp khi hết giờ</t>
-        </is>
-      </c>
-      <c r="E111" s="4" t="inlineStr">
-        <is>
-          <t>Lưu lần chọn đầu/cuối, số lần lưu từng câu; giới hạn thời gian; lượt hết giờ tự nộp</t>
-        </is>
-      </c>
+          <t>test_tim_dung_slide[T\u1ec7p nh\u1eadt k\xfd giao t\xe1c (.ldf) trong SQL Server \u0111\u01b0\u1ee3c d\xf9ng ch\u1ee7 y\u1ebfu \u0111\u1ec3 ph\u1ee5c h\u1ed3i-Slide b\xe0i gi\u1ea3ng \u2013 Ch\u01b0\u01a1ng 1-4]</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr"/>
+      <c r="E111" s="4" t="inlineStr"/>
       <c r="F111" s="5" t="inlineStr">
         <is>
           <t>ĐẠT</t>
@@ -5123,7 +5168,7 @@
       </c>
       <c r="H111" s="4" t="inlineStr">
         <is>
-          <t>test_timing::test_sync_stores_answer_times</t>
+          <t>test_hoc_lieu_rag::test_tim_dung_slide[T\u1ec7p nh\u1eadt k\xfd giao t\xe1c (.ldf) trong SQL Server \u0111\u01b0\u1ee3c d\xf9ng ch\u1ee7 y\u1ebfu \u0111\u1ec3 ph\u1ee5c h\u1ed3i-Slide b\xe0i gi\u1ea3ng \u2013 Ch\u01b0\u01a1ng 1-4]</t>
         </is>
       </c>
       <c r="I111" s="4" t="inlineStr"/>
@@ -5134,35 +5179,27 @@
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>13. Thời gian làm bài &amp; cảnh báo bất thường</t>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>Cảnh báo SV chọn đại / chọn xong để hết giờ</t>
-        </is>
-      </c>
-      <c r="D112" s="4" t="inlineStr">
-        <is>
-          <t>Dữ liệu có 2 SV chọn ~20 câu trong 1 phút và 2 SV chọn xong không nộp chờ hết giờ</t>
-        </is>
-      </c>
-      <c r="E112" s="4" t="inlineStr">
-        <is>
-          <t>Đúng 4 SV bị cảnh báo đúng loại; SV bình thường không bị gắn cờ; số cảnh báo hiện ở danh sách bài KT</t>
-        </is>
-      </c>
+          <t>test_tim_dung_slide[Trong trigger AFTER UPDATE b\u1ea3ng t\u1ea1m n\xe0o ch\u1ee9a gi\xe1 tr\u1ecb C\u0168 c\u1ee7a c\xe1c d\xf2ng b\u1ecb c\u1eadp nh\u1eadt-Slide b\xe0i gi\u1ea3ng \u2013 Ch\u01b0\u01a1ng 3-1]</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr"/>
+      <c r="E112" s="4" t="inlineStr"/>
       <c r="F112" s="5" t="inlineStr">
         <is>
           <t>ĐẠT</t>
         </is>
       </c>
       <c r="G112" s="4" t="n">
-        <v>0.21</v>
+        <v>0.01</v>
       </c>
       <c r="H112" s="4" t="inlineStr">
         <is>
-          <t>test_timing::test_timing_report_flags_planted_students</t>
+          <t>test_hoc_lieu_rag::test_tim_dung_slide[Trong trigger AFTER UPDATE b\u1ea3ng t\u1ea1m n\xe0o ch\u1ee9a gi\xe1 tr\u1ecb C\u0168 c\u1ee7a c\xe1c d\xf2ng b\u1ecb c\u1eadp nh\u1eadt-Slide b\xe0i gi\u1ea3ng \u2013 Ch\u01b0\u01a1ng 3-1]</t>
         </is>
       </c>
       <c r="I112" s="4" t="inlineStr"/>
@@ -5173,38 +5210,637 @@
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>13. Thời gian làm bài &amp; cảnh báo bất thường</t>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>Đổi ngưỡng, diễn biến từng SV, xuất Excel</t>
-        </is>
-      </c>
-      <c r="D113" s="4" t="inlineStr">
-        <is>
-          <t>Gửi ngưỡng tùy chỉnh / sai; xem diễn biến 1 SV; tải Excel; bài giấy</t>
-        </is>
-      </c>
-      <c r="E113" s="4" t="inlineStr">
-        <is>
-          <t>Kết quả theo ngưỡng; ngưỡng sai 422; SV không làm 404; Excel 2 sheet; bài giấy báo không áp dụng</t>
-        </is>
-      </c>
+          <t>test_tim_dung_slide[Hai giao t\xe1c gi\u1eef kh\xf3a ch\u1edd nhau deadlock ch\u1ecdn n\u1ea1n nh\xe2n victim-Slide b\xe0i gi\u1ea3ng \u2013 Ch\u01b0\u01a1ng 4-4]</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr"/>
+      <c r="E113" s="4" t="inlineStr"/>
       <c r="F113" s="5" t="inlineStr">
         <is>
           <t>ĐẠT</t>
         </is>
       </c>
       <c r="G113" s="4" t="n">
-        <v>0.2</v>
+        <v>0.01</v>
       </c>
       <c r="H113" s="4" t="inlineStr">
         <is>
-          <t>test_timing::test_timing_thresholds_timeline_and_export</t>
+          <t>test_hoc_lieu_rag::test_tim_dung_slide[Hai giao t\xe1c gi\u1eef kh\xf3a ch\u1edd nhau deadlock ch\u1ecdn n\u1ea1n nh\xe2n victim-Slide b\xe0i gi\u1ea3ng \u2013 Ch\u01b0\u01a1ng 4-4]</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C114" s="4" t="inlineStr">
+        <is>
+          <t>test_tim_dung_slide[M\u1ed7i b\u1ea3ng trong SQL Server c\xf3 t\u1ed1i \u0111a bao nhi\xeau ch\u1ec9 m\u1ee5c clustered-Slide b\xe0i gi\u1ea3ng \u2013 Ch\u01b0\u01a1ng 5-1]</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr"/>
+      <c r="E114" s="4" t="inlineStr"/>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G114" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H114" s="4" t="inlineStr">
+        <is>
+          <t>test_hoc_lieu_rag::test_tim_dung_slide[M\u1ed7i b\u1ea3ng trong SQL Server c\xf3 t\u1ed1i \u0111a bao nhi\xeau ch\u1ec9 m\u1ee5c clustered-Slide b\xe0i gi\u1ea3ng \u2013 Ch\u01b0\u01a1ng 5-1]</t>
+        </is>
+      </c>
+      <c r="I114" s="4" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>test_tim_dung_slide[B\u1ea3n sao l\u01b0u differential ch\u1ee9a g\xec-Slide b\xe0i gi\u1ea3ng \u2013 Ch\u01b0\u01a1ng 6-3]</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr"/>
+      <c r="E115" s="4" t="inlineStr"/>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G115" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H115" s="4" t="inlineStr">
+        <is>
+          <t>test_hoc_lieu_rag::test_tim_dung_slide[B\u1ea3n sao l\u01b0u differential ch\u1ee9a g\xec-Slide b\xe0i gi\u1ea3ng \u2013 Ch\u01b0\u01a1ng 6-3]</t>
+        </is>
+      </c>
+      <c r="I115" s="4" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C116" s="4" t="inlineStr">
+        <is>
+          <t>Câu ngoài phạm vi học liệu</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>Tìm một câu hỏi không liên quan môn</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="inlineStr">
+        <is>
+          <t>Kết quả rỗng, không gợi ý bừa</t>
+        </is>
+      </c>
+      <c r="F116" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G116" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H116" s="4" t="inlineStr">
+        <is>
+          <t>test_hoc_lieu_rag::test_cau_ngoai_pham_vi_khong_goi_y</t>
+        </is>
+      </c>
+      <c r="I116" s="4" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>Chỉ tìm trong học liệu của đúng môn</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>Tải tài liệu vào môn khác rồi tìm ở cả hai môn</t>
+        </is>
+      </c>
+      <c r="E117" s="4" t="inlineStr">
+        <is>
+          <t>Mỗi môn chỉ thấy tài liệu của mình</t>
+        </is>
+      </c>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G117" s="4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H117" s="4" t="inlineStr">
+        <is>
+          <t>test_hoc_lieu_rag::test_chi_tim_trong_hoc_lieu_cua_dung_khoa</t>
+        </is>
+      </c>
+      <c r="I117" s="4" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="4" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C118" s="4" t="inlineStr">
+        <is>
+          <t>Tải học liệu DOCX/TXT và các lỗi</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>Tải DOCX, TXT; tệp .exe, tệp rỗng, loại học liệu sai</t>
+        </is>
+      </c>
+      <c r="E118" s="4" t="inlineStr">
+        <is>
+          <t>201 và có chỉ mục; 422 cho các trường hợp lỗi</t>
+        </is>
+      </c>
+      <c r="F118" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G118" s="4" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H118" s="4" t="inlineStr">
+        <is>
+          <t>test_hoc_lieu_rag::test_tai_len_docx_txt_va_loi</t>
+        </is>
+      </c>
+      <c r="I118" s="4" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>Gợi ý đọc cho sinh viên làm sai</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>Dữ liệu kết quả gửi Moodle của bài đã phân tích</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="inlineStr">
+        <is>
+          <t>Mỗi SV có danh sách trang/slide thuộc học liệu của môn; không lộ mã câu hỏi</t>
+        </is>
+      </c>
+      <c r="F119" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G119" s="4" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H119" s="4" t="inlineStr">
+        <is>
+          <t>test_hoc_lieu_rag::test_goi_y_doc_cho_sv_lam_sai</t>
+        </is>
+      </c>
+      <c r="I119" s="4" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C120" s="4" t="inlineStr">
+        <is>
+          <t>Tạo lại gợi ý đọc</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>Thêm học liệu rồi gọi readings/rebuild; bài không tồn tại</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="inlineStr">
+        <is>
+          <t>Hầu hết SV có gợi ý; 404</t>
+        </is>
+      </c>
+      <c r="F120" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G120" s="4" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="H120" s="4" t="inlineStr">
+        <is>
+          <t>test_hoc_lieu_rag::test_tai_tao_goi_y_sau_khi_them_hoc_lieu</t>
+        </is>
+      </c>
+      <c r="I120" s="4" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>Lấy học liệu từ khóa học Moodle</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>Moodle giả lập trả danh sách tệp; lấy lần 2; đẩy ngược tệp lấy từ Moodle</t>
+        </is>
+      </c>
+      <c r="E121" s="4" t="inlineStr">
+        <is>
+          <t>Thêm tệp mới, không trùng; 409 khi đẩy ngược</t>
+        </is>
+      </c>
+      <c r="F121" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G121" s="4" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H121" s="4" t="inlineStr">
+        <is>
+          <t>test_hoc_lieu_rag::test_lay_hoc_lieu_tu_moodle_ve</t>
+        </is>
+      </c>
+      <c r="I121" s="4" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>Đưa học liệu lên Moodle</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>Gọi local_clo_add_resource (giả lập)</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>Nhận course module id; lưu lại để SV mở được</t>
+        </is>
+      </c>
+      <c r="F122" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G122" s="4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H122" s="4" t="inlineStr">
+        <is>
+          <t>test_hoc_lieu_rag::test_day_hoc_lieu_len_moodle</t>
+        </is>
+      </c>
+      <c r="I122" s="4" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>Moodle báo lỗi khi đồng bộ học liệu</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>Web Service giả lập trả lỗi</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="inlineStr">
+        <is>
+          <t>502 kèm thông báo</t>
+        </is>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G123" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H123" s="4" t="inlineStr">
+        <is>
+          <t>test_hoc_lieu_rag::test_moodle_loi_tra_502</t>
+        </is>
+      </c>
+      <c r="I123" s="4" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C124" s="4" t="inlineStr">
+        <is>
+          <t>Gợi ý đọc ở trang Ôn tập</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>Tổng quan Ôn tập của lớp</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="inlineStr">
+        <is>
+          <t>Mỗi SV yếu và mỗi chương có danh sách trang nên đọc</t>
+        </is>
+      </c>
+      <c r="F124" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G124" s="4" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H124" s="4" t="inlineStr">
+        <is>
+          <t>test_hoc_lieu_rag::test_on_tap_co_goi_y_doc</t>
+        </is>
+      </c>
+      <c r="I124" s="4" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>Xem lại trang, tải tệp gốc, lập lại chỉ mục</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>Mở trang 2 của slide chương 4; trang không có; tải tệp; lập lại chỉ mục</t>
+        </is>
+      </c>
+      <c r="E125" s="4" t="inlineStr">
+        <is>
+          <t>Trang đúng nội dung; 404; tệp PPTX; số trang không đổi</t>
+        </is>
+      </c>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G125" s="4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H125" s="4" t="inlineStr">
+        <is>
+          <t>test_hoc_lieu_rag::test_xem_tep_goc_trang_va_lap_lai_chi_muc</t>
+        </is>
+      </c>
+      <c r="I125" s="4" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="4" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C126" s="4" t="inlineStr">
+        <is>
+          <t>test_lay_ve_khong_trung_voi_tep_da_day_len</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr"/>
+      <c r="E126" s="4" t="inlineStr"/>
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G126" s="4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H126" s="4" t="inlineStr">
+        <is>
+          <t>test_hoc_lieu_rag::test_lay_ve_khong_trung_voi_tep_da_day_len</t>
+        </is>
+      </c>
+      <c r="I126" s="4" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t>test_demo_syllabus_approved</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr"/>
+      <c r="E127" s="4" t="inlineStr"/>
+      <c r="F127" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G127" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H127" s="4" t="inlineStr">
+        <is>
+          <t>test_syllabus_versions::test_demo_syllabus_approved</t>
+        </is>
+      </c>
+      <c r="I127" s="4" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="4" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t>test_syllabus_version_flow</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr"/>
+      <c r="E128" s="4" t="inlineStr"/>
+      <c r="F128" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G128" s="4" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="H128" s="4" t="inlineStr">
+        <is>
+          <t>test_syllabus_versions::test_syllabus_version_flow</t>
+        </is>
+      </c>
+      <c r="I128" s="4" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C129" s="4" t="inlineStr">
+        <is>
+          <t>test_outline_detail</t>
+        </is>
+      </c>
+      <c r="D129" s="4" t="inlineStr"/>
+      <c r="E129" s="4" t="inlineStr"/>
+      <c r="F129" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G129" s="4" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H129" s="4" t="inlineStr">
+        <is>
+          <t>test_syllabus_versions::test_outline_detail</t>
+        </is>
+      </c>
+      <c r="I129" s="4" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="4" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t>14. Học liệu và gợi ý đọc (RAG theo trang)</t>
+        </is>
+      </c>
+      <c r="C130" s="4" t="inlineStr">
+        <is>
+          <t>test_new_course_without_syllabus</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr"/>
+      <c r="E130" s="4" t="inlineStr"/>
+      <c r="F130" s="5" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="G130" s="4" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H130" s="4" t="inlineStr">
+        <is>
+          <t>test_syllabus_versions::test_new_course_without_syllabus</t>
+        </is>
+      </c>
+      <c r="I130" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5217,7 +5853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G139"/>
+  <dimension ref="A1:G149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8202,7 +8838,7 @@
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>test_overview_theo_chuong_va_loc_chuong, test_remedial_flow</t>
+          <t>test_on_tap_co_goi_y_doc, test_overview_theo_chuong_va_loc_chuong, test_remedial_flow</t>
         </is>
       </c>
     </row>
@@ -9252,7 +9888,7 @@
       </c>
       <c r="G115" s="4" t="inlineStr">
         <is>
-          <t>test_results_for_moodle</t>
+          <t>test_goi_y_doc_cho_sv_lam_sai, test_results_for_moodle</t>
         </is>
       </c>
     </row>
@@ -10037,17 +10673,17 @@
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>/api/health</t>
+          <t>/api/courses/{cid}/materials</t>
         </is>
       </c>
       <c r="D138" s="4" t="inlineStr">
         <is>
-          <t>Hệ thống</t>
+          <t>Học liệu và gợi ý đọc (RAG)</t>
         </is>
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra dịch vụ</t>
+          <t>list_materials</t>
         </is>
       </c>
       <c r="F138" s="5" t="inlineStr">
@@ -10057,7 +10693,7 @@
       </c>
       <c r="G138" s="4" t="inlineStr">
         <is>
-          <t>test_auth_me_and_catalogs</t>
+          <t>test_day_hoc_lieu_len_moodle, test_lay_hoc_lieu_tu_moodle_ve, test_lay_ve_khong_trung_voi_tep_da_day_len, test_seed_co_hoc_lieu, test_tai_len_docx_txt_va_loi, test_xem_tep_goc_trang_va_lap_lai_chi_muc</t>
         </is>
       </c>
     </row>
@@ -10067,30 +10703,380 @@
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>/api/courses/{cid}/materials</t>
+        </is>
+      </c>
+      <c r="D139" s="4" t="inlineStr">
+        <is>
+          <t>Học liệu và gợi ý đọc (RAG)</t>
+        </is>
+      </c>
+      <c r="E139" s="4" t="inlineStr">
+        <is>
+          <t>upload_material</t>
+        </is>
+      </c>
+      <c r="F139" s="5" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G139" s="4" t="inlineStr">
+        <is>
+          <t>test_day_hoc_lieu_len_moodle, test_lay_ve_khong_trung_voi_tep_da_day_len, test_tai_len_docx_txt_va_loi</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="4" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="C140" s="4" t="inlineStr">
+        <is>
+          <t>/api/materials/{mid}</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>Học liệu và gợi ý đọc (RAG)</t>
+        </is>
+      </c>
+      <c r="E140" s="4" t="inlineStr">
+        <is>
+          <t>delete_material</t>
+        </is>
+      </c>
+      <c r="F140" s="5" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G140" s="4" t="inlineStr">
+        <is>
+          <t>test_chi_tim_trong_hoc_lieu_cua_dung_khoa, test_day_hoc_lieu_len_moodle, test_lay_hoc_lieu_tu_moodle_ve, test_lay_ve_khong_trung_voi_tep_da_day_len, test_tai_len_docx_txt_va_loi</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C141" s="4" t="inlineStr">
+        <is>
+          <t>/api/materials/{mid}/reindex</t>
+        </is>
+      </c>
+      <c r="D141" s="4" t="inlineStr">
+        <is>
+          <t>Học liệu và gợi ý đọc (RAG)</t>
+        </is>
+      </c>
+      <c r="E141" s="4" t="inlineStr">
+        <is>
+          <t>reindex</t>
+        </is>
+      </c>
+      <c r="F141" s="5" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G141" s="4" t="inlineStr">
+        <is>
+          <t>test_xem_tep_goc_trang_va_lap_lai_chi_muc</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="4" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C139" s="4" t="inlineStr">
+      <c r="C142" s="4" t="inlineStr">
+        <is>
+          <t>/api/materials/{mid}/file</t>
+        </is>
+      </c>
+      <c r="D142" s="4" t="inlineStr">
+        <is>
+          <t>Học liệu và gợi ý đọc (RAG)</t>
+        </is>
+      </c>
+      <c r="E142" s="4" t="inlineStr">
+        <is>
+          <t>download</t>
+        </is>
+      </c>
+      <c r="F142" s="5" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G142" s="4" t="inlineStr">
+        <is>
+          <t>test_xem_tep_goc_trang_va_lap_lai_chi_muc</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="4" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C143" s="4" t="inlineStr">
+        <is>
+          <t>/api/materials/{mid}/pages/{page}</t>
+        </is>
+      </c>
+      <c r="D143" s="4" t="inlineStr">
+        <is>
+          <t>Học liệu và gợi ý đọc (RAG)</t>
+        </is>
+      </c>
+      <c r="E143" s="4" t="inlineStr">
+        <is>
+          <t>page_text</t>
+        </is>
+      </c>
+      <c r="F143" s="5" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G143" s="4" t="inlineStr">
+        <is>
+          <t>test_xem_tep_goc_trang_va_lap_lai_chi_muc</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="4" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C144" s="4" t="inlineStr">
+        <is>
+          <t>/api/courses/{cid}/materials/search</t>
+        </is>
+      </c>
+      <c r="D144" s="4" t="inlineStr">
+        <is>
+          <t>Học liệu và gợi ý đọc (RAG)</t>
+        </is>
+      </c>
+      <c r="E144" s="4" t="inlineStr">
+        <is>
+          <t>Thử truy xuất: gõ câu hỏi/thuật ngữ → trang/slide của học liệu thuộc học phần này.</t>
+        </is>
+      </c>
+      <c r="F144" s="5" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G144" s="4" t="inlineStr">
+        <is>
+          <t>test_cau_ngoai_pham_vi_khong_goi_y, test_chi_tim_trong_hoc_lieu_cua_dung_khoa, test_lay_hoc_lieu_tu_moodle_ve, test_tai_len_docx_txt_va_loi, test_tim_dung_slide[B\u1ea3n, test_tim_dung_slide[Hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="4" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C145" s="4" t="inlineStr">
+        <is>
+          <t>/api/exams/{eid}/readings/rebuild</t>
+        </is>
+      </c>
+      <c r="D145" s="4" t="inlineStr">
+        <is>
+          <t>Học liệu và gợi ý đọc (RAG)</t>
+        </is>
+      </c>
+      <c r="E145" s="4" t="inlineStr">
+        <is>
+          <t>Tạo lại gợi ý đọc của cả bài KT từ học liệu hiện có (dùng sau khi tải thêm học liệu, không cần phân tích lại).</t>
+        </is>
+      </c>
+      <c r="F145" s="5" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G145" s="4" t="inlineStr">
+        <is>
+          <t>test_tai_tao_goi_y_sau_khi_them_hoc_lieu</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="4" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C146" s="4" t="inlineStr">
+        <is>
+          <t>/api/courses/{cid}/materials/sync-moodle</t>
+        </is>
+      </c>
+      <c r="D146" s="4" t="inlineStr">
+        <is>
+          <t>Học liệu và gợi ý đọc (RAG)</t>
+        </is>
+      </c>
+      <c r="E146" s="4" t="inlineStr">
+        <is>
+          <t>Lấy học liệu đã có trong khóa học Moodle (hoạt động Tệp/Thư mục: PDF, PPTX, DOCX, TXT, MD) về lập chỉ mục.</t>
+        </is>
+      </c>
+      <c r="F146" s="5" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G146" s="4" t="inlineStr">
+        <is>
+          <t>test_lay_hoc_lieu_tu_moodle_ve, test_lay_ve_khong_trung_voi_tep_da_day_len</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="4" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>/api/materials/{mid}/push-moodle</t>
+        </is>
+      </c>
+      <c r="D147" s="4" t="inlineStr">
+        <is>
+          <t>Học liệu và gợi ý đọc (RAG)</t>
+        </is>
+      </c>
+      <c r="E147" s="4" t="inlineStr">
+        <is>
+          <t>Đẩy học liệu lên khóa học Moodle thành hoạt động Tệp để sinh viên xem ngay trên Moodle.</t>
+        </is>
+      </c>
+      <c r="F147" s="5" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G147" s="4" t="inlineStr">
+        <is>
+          <t>test_day_hoc_lieu_len_moodle, test_lay_ve_khong_trung_voi_tep_da_day_len</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="4" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C148" s="4" t="inlineStr">
+        <is>
+          <t>/api/health</t>
+        </is>
+      </c>
+      <c r="D148" s="4" t="inlineStr">
+        <is>
+          <t>Hệ thống</t>
+        </is>
+      </c>
+      <c r="E148" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra dịch vụ</t>
+        </is>
+      </c>
+      <c r="F148" s="5" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G148" s="4" t="inlineStr">
+        <is>
+          <t>test_auth_me_and_catalogs</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="4" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C149" s="4" t="inlineStr">
         <is>
           <t>/api/public-config</t>
         </is>
       </c>
-      <c r="D139" s="4" t="inlineStr">
+      <c r="D149" s="4" t="inlineStr">
         <is>
           <t>Hệ thống</t>
         </is>
       </c>
-      <c r="E139" s="4" t="inlineStr">
+      <c r="E149" s="4" t="inlineStr">
         <is>
           <t>Cấu hình công khai cho giao diện</t>
         </is>
       </c>
-      <c r="F139" s="5" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="G139" s="4" t="inlineStr">
+      <c r="F149" s="5" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G149" s="4" t="inlineStr">
         <is>
           <t>test_auth_me_and_catalogs</t>
         </is>
@@ -10107,7 +11093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11242,21 +12228,166 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Thời gian làm bài &amp; cảnh báo</t>
+          <t>Học liệu của môn</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Bài Thi cuối kỳ (Moodle) &gt; thẻ 'Thời gian làm bài'; bấm 'Diễn biến' của SV 22130017; đổi ngưỡng giây/câu rồi Áp dụng; Xuất Excel</t>
+          <t>Trang môn học &gt; tab Học liệu: tải lên slide/giáo trình; bấm Lập lại chỉ mục; gõ một câu hỏi vào ô tìm thử</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>4 SV bị cảnh báo (2 làm quá nhanh, 2 để hết giờ tự nộp); biểu đồ từng câu; danh sách đổi theo ngưỡng; tải được Excel</t>
+          <t>Danh sách có số trang đã lập chỉ mục; kết quả tìm là trang/slide đúng kèm độ khớp và đoạn trích</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr"/>
       <c r="G39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>GD-39</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>GV</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Gợi ý đọc trong hồ sơ sinh viên</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Lớp học phần &gt; Thống kê &gt; chọn một sinh viên</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Mục Cần đọc lại ở đâu: tên tài liệu, trang/slide, các câu làm sai dẫn tới đó</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>GD-40</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>GV</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Gợi ý đọc ở trang Ôn tập</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Lớp học phần &gt; Ôn tập &gt; tab Theo chương</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Cột Nên đọc lại cho từng chương; tích chọn chương rồi tạo bài kiểm tra cho nhóm vẫn dùng được</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>GD-41</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>GV</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Đồng bộ học liệu với Moodle</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Tab Học liệu: Đưa lên Moodle một tệp; Lấy từ Moodle</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Tệp xuất hiện trong khóa học Moodle; tệp mới trên Moodle được lấy về, không trùng</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>GD-42</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Gợi ý đọc trên Moodle</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Đăng nhập Moodle bằng tài khoản sinh viên &gt; khóa học &gt; Kết quả phân tích CĐR</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Mục Nên đọc lại ở đâu liệt kê trang/slide; bấm tên tài liệu mở được tài nguyên trong khóa học</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>GD-43</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>GV</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Thời gian làm bài &amp; cảnh báo</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Bài Thi cuối kỳ (Moodle) &gt; thẻ 'Thời gian làm bài'; bấm 'Diễn biến' của SV 22130017; đổi ngưỡng giây/câu rồi Áp dụng; Xuất Excel</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>4 SV bị cảnh báo (2 làm quá nhanh, 2 để hết giờ tự nộp); biểu đồ từng câu; danh sách đổi theo ngưỡng; tải được Excel</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>